<commit_message>
fix: 同步 root files 目录与 build_web 自动复制逻辑，修复 GitHub Pages 404 调取 Excel 盘源失败
</commit_message>
<xml_diff>
--- a/files/九龙-九龙塘-皇廷汇.xlsx
+++ b/files/九龙-九龙塘-皇廷汇.xlsx
@@ -990,7 +990,7 @@
         <is>
           <t>A号屋
 10718呎 (4+房)
-(24年-03月)
+(24年-03月-21日)
 $3.40亿
 $31,722/呎</t>
         </is>
@@ -999,7 +999,7 @@
         <is>
           <t>B号屋
 5845呎 (4+房)
-(23年-08月)
+(23年-08月-17日)
 $2.55亿
 $43,593/呎</t>
         </is>
@@ -1017,7 +1017,7 @@
         <is>
           <t>喇沙利道（独立屋）
 7338呎 (4+房)
-(17年-04月)
+(17年-04月-06日)
 $3.09亿
 $42,082/呎</t>
         </is>

</xml_diff>